<commit_message>
excel file info page added
</commit_message>
<xml_diff>
--- a/Results/ESM_17_Cooling_rates_single_track_AM_Bench_2022_double_and_single_conical.xlsx
+++ b/Results/ESM_17_Cooling_rates_single_track_AM_Bench_2022_double_and_single_conical.xlsx
@@ -1,81 +1,192 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University of Dayton\Reseach in UD\new_graphs_july\Final results\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF064C6-F92B-4B35-91BA-0C8411B60E25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Double_conical" sheetId="4" r:id="rId1"/>
-    <sheet name="Single_conical" sheetId="5" r:id="rId2"/>
+    <sheet sheetId="1" name="Double_conical" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Single_conical" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="info" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
+  <si>
+    <t>point</t>
+  </si>
+  <si>
+    <t>SCR (C/s)</t>
+  </si>
+  <si>
+    <t>TCR(C/s)</t>
+  </si>
+  <si>
+    <t>LCR(C/s)</t>
+  </si>
+  <si>
+    <t>TAM(s)</t>
+  </si>
   <si>
     <t>sim avg</t>
   </si>
   <si>
-    <t>TCR(C/s)</t>
-  </si>
-  <si>
-    <t>SCR (C/s)</t>
-  </si>
-  <si>
-    <t>LCR(C/s)</t>
-  </si>
-  <si>
-    <t>TAM(s)</t>
-  </si>
-  <si>
-    <t>point</t>
+    <t>Simulation / Data Information</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Information</t>
+  </si>
+  <si>
+    <t>Online Resource</t>
+  </si>
+  <si>
+    <t>ESM_17</t>
+  </si>
+  <si>
+    <t>Benchmark</t>
+  </si>
+  <si>
+    <t>NIST AM-Bench 2022</t>
+  </si>
+  <si>
+    <t>Simulation case</t>
+  </si>
+  <si>
+    <t>Single-track Case 0</t>
+  </si>
+  <si>
+    <t>Heat-source models</t>
+  </si>
+  <si>
+    <t>Single-conical and Double Conical Heat Source (DCHS)</t>
+  </si>
+  <si>
+    <t>Track length</t>
+  </si>
+  <si>
+    <t>2 mm</t>
+  </si>
+  <si>
+    <t>Laser power</t>
+  </si>
+  <si>
+    <t>285 W</t>
+  </si>
+  <si>
+    <t>Scan speed</t>
+  </si>
+  <si>
+    <t>960 mm/s</t>
+  </si>
+  <si>
+    <t>Laser spot diameter</t>
+  </si>
+  <si>
+    <t>67 µm</t>
+  </si>
+  <si>
+    <t>Data included</t>
+  </si>
+  <si>
+    <t>Solid cooling rate (SCR), transitional cooling rate (TCR), liquid cooling rate (LCR), and time above melt (TAM) at multiple monitoring points</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>Cooling rates: °C/s; TAM: s</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Thermal-metric validation of the AM-Bench 2022 single-track model and comparison of the single-conical and DCHS models</t>
+  </si>
+  <si>
+    <t>Related simulation videos</t>
+  </si>
+  <si>
+    <t>ESM_1 and ESM_2</t>
+  </si>
+  <si>
+    <t>Related temperature-history videos</t>
+  </si>
+  <si>
+    <t>ESM_8 and ESM_9</t>
+  </si>
+  <si>
+    <t>Related manuscript section</t>
+  </si>
+  <si>
+    <t>AM-Bench 2022 single-track validation</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>The workbook provides point-wise thermal metrics obtained from the simulated temperature histories for both heat-source models.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="5" x14ac:knownFonts="1">
+    <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="14"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+      <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -90,9 +201,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -121,44 +244,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -188,12 +311,12 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -232,159 +355,221 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF23DA4F-6860-4E14-85D0-6B0605EAF0B7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E27"/>
-  <sheetFormatPr defaultColWidth="11.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
       </c>
       <c r="D1" t="s">
         <v>3</v>
@@ -393,7 +578,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -407,10 +592,10 @@
         <v>-430100</v>
       </c>
       <c r="E2">
-        <v>1.1800000000000001E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -424,10 +609,10 @@
         <v>-451500</v>
       </c>
       <c r="E3">
-        <v>1.17E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -441,10 +626,10 @@
         <v>-439100</v>
       </c>
       <c r="E4">
-        <v>1.15E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -458,10 +643,10 @@
         <v>-451500</v>
       </c>
       <c r="E5">
-        <v>1.17E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -475,10 +660,10 @@
         <v>-439000</v>
       </c>
       <c r="E6">
-        <v>1.15E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -492,10 +677,10 @@
         <v>-451300</v>
       </c>
       <c r="E7" s="1">
-        <v>1.1800000000000001E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00118</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -509,10 +694,10 @@
         <v>-438900</v>
       </c>
       <c r="E8" s="1">
-        <v>1.17E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -526,10 +711,10 @@
         <v>-444400</v>
       </c>
       <c r="E9">
-        <v>1.15E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -543,10 +728,10 @@
         <v>-438900</v>
       </c>
       <c r="E10">
-        <v>1.17E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -560,10 +745,10 @@
         <v>-444400</v>
       </c>
       <c r="E11">
-        <v>1.15E-3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -577,10 +762,10 @@
         <v>-437800</v>
       </c>
       <c r="E12">
-        <v>1.1800000000000001E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00118</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -594,10 +779,10 @@
         <v>-443500</v>
       </c>
       <c r="E13">
-        <v>1.17E-3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -611,10 +796,10 @@
         <v>-446400</v>
       </c>
       <c r="E14">
-        <v>1.15E-3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -628,10 +813,10 @@
         <v>-443500</v>
       </c>
       <c r="E15">
-        <v>1.17E-3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -645,10 +830,10 @@
         <v>-446400</v>
       </c>
       <c r="E16">
-        <v>1.15E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -662,10 +847,10 @@
         <v>-443200</v>
       </c>
       <c r="E17">
-        <v>1.1800000000000001E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00118</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
@@ -679,10 +864,10 @@
         <v>-448700</v>
       </c>
       <c r="E18">
-        <v>1.17E-3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
@@ -696,10 +881,10 @@
         <v>-451600</v>
       </c>
       <c r="E19">
-        <v>1.15E-3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
@@ -713,10 +898,10 @@
         <v>-448700</v>
       </c>
       <c r="E20">
-        <v>1.17E-3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
@@ -730,10 +915,10 @@
         <v>-451600</v>
       </c>
       <c r="E21">
-        <v>1.15E-3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
@@ -747,10 +932,10 @@
         <v>-421900</v>
       </c>
       <c r="E22">
-        <v>1.1800000000000001E-3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>21</v>
       </c>
@@ -764,10 +949,10 @@
         <v>-443700</v>
       </c>
       <c r="E23">
-        <v>1.17E-3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>22</v>
       </c>
@@ -781,10 +966,10 @@
         <v>-449300</v>
       </c>
       <c r="E24">
-        <v>1.15E-3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>23</v>
       </c>
@@ -798,10 +983,10 @@
         <v>-443700</v>
       </c>
       <c r="E25">
-        <v>1.17E-3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00117</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>24</v>
       </c>
@@ -815,54 +1000,53 @@
         <v>-449200</v>
       </c>
       <c r="E26">
-        <v>1.15E-3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00115</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B27" s="1">
         <f>AVERAGE(B2:B26)</f>
-        <v>-887080</v>
       </c>
       <c r="C27" s="1">
-        <f t="shared" ref="C27:E27" si="0">AVERAGE(C2:C26)</f>
-        <v>-260208</v>
+        <f>AVERAGE(C2:C26)</f>
       </c>
       <c r="D27" s="1">
-        <f t="shared" si="0"/>
-        <v>-443932</v>
+        <f>AVERAGE(D2:D26)</f>
       </c>
       <c r="E27" s="1">
-        <f t="shared" si="0"/>
-        <v>1.1640000000000003E-3</v>
+        <f>AVERAGE(E2:E26)</f>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4785560D-E935-4419-A57A-1A3275D17045}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="2" max="2" width="13.77734375" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
+    <col min="1" max="1" width="13.571428571428571" customWidth="1"/>
+    <col min="2" max="2" width="13.714285714285714" customWidth="1"/>
+    <col min="3" max="3" width="13.285714285714286" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
       </c>
       <c r="D1" t="s">
         <v>3</v>
@@ -871,7 +1055,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -885,10 +1069,10 @@
         <v>-389500</v>
       </c>
       <c r="E2">
-        <v>1.33E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -902,10 +1086,10 @@
         <v>-393900</v>
       </c>
       <c r="E3">
-        <v>1.31E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00131</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -919,10 +1103,10 @@
         <v>-395900</v>
       </c>
       <c r="E4">
-        <v>1.2999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.0013</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -936,10 +1120,10 @@
         <v>-393900</v>
       </c>
       <c r="E5">
-        <v>1.31E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00131</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -953,10 +1137,10 @@
         <v>-395900</v>
       </c>
       <c r="E6">
-        <v>1.2999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.0013</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -970,10 +1154,10 @@
         <v>-378800</v>
       </c>
       <c r="E7" s="1">
-        <v>1.33E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -987,10 +1171,10 @@
         <v>-395400</v>
       </c>
       <c r="E8" s="1">
-        <v>1.31E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00131</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -1004,10 +1188,10 @@
         <v>-399700</v>
       </c>
       <c r="E9">
-        <v>1.2999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.0013</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1021,10 +1205,10 @@
         <v>-395400</v>
       </c>
       <c r="E10">
-        <v>1.31E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00131</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -1038,10 +1222,10 @@
         <v>-399700</v>
       </c>
       <c r="E11">
-        <v>1.2999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.0013</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1055,10 +1239,10 @@
         <v>-395000</v>
       </c>
       <c r="E12">
-        <v>1.33E-3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -1072,10 +1256,10 @@
         <v>-385200</v>
       </c>
       <c r="E13">
-        <v>1.31E-3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00131</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -1089,10 +1273,10 @@
         <v>-389500</v>
       </c>
       <c r="E14">
-        <v>1.2999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.0013</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -1106,10 +1290,10 @@
         <v>-385200</v>
       </c>
       <c r="E15">
-        <v>1.31E-3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00131</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -1123,10 +1307,10 @@
         <v>-389500</v>
       </c>
       <c r="E16">
-        <v>1.2999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.0013</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -1140,10 +1324,10 @@
         <v>-372800</v>
       </c>
       <c r="E17">
-        <v>1.33E-3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00133</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
@@ -1157,10 +1341,10 @@
         <v>-389600</v>
       </c>
       <c r="E18">
-        <v>1.31E-3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
@@ -1174,10 +1358,10 @@
         <v>-394000</v>
       </c>
       <c r="E19">
-        <v>1.2999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.0013</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
@@ -1191,10 +1375,10 @@
         <v>-389600</v>
       </c>
       <c r="E20">
-        <v>1.31E-3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00131</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
@@ -1208,10 +1392,10 @@
         <v>-393900</v>
       </c>
       <c r="E21">
-        <v>1.2999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.0013</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
@@ -1225,10 +1409,10 @@
         <v>-383200</v>
       </c>
       <c r="E22">
-        <v>1.33E-3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00133</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>21</v>
       </c>
@@ -1242,10 +1426,10 @@
         <v>-387800</v>
       </c>
       <c r="E23">
-        <v>1.31E-3</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00131</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>22</v>
       </c>
@@ -1259,10 +1443,10 @@
         <v>-389800</v>
       </c>
       <c r="E24">
-        <v>1.2999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.0013</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>23</v>
       </c>
@@ -1276,10 +1460,10 @@
         <v>-387800</v>
       </c>
       <c r="E25">
-        <v>1.31E-3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.00131</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>24</v>
       </c>
@@ -1293,31 +1477,181 @@
         <v>-389800</v>
       </c>
       <c r="E26">
-        <v>1.2999999999999999E-3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.0013</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B27" s="1">
         <f>AVERAGE(B2:B26)</f>
-        <v>-786540</v>
       </c>
       <c r="C27" s="1">
-        <f t="shared" ref="C27:E27" si="0">AVERAGE(C2:C26)</f>
-        <v>-226748</v>
+        <f>AVERAGE(C2:C26)</f>
       </c>
       <c r="D27" s="1">
-        <f t="shared" si="0"/>
-        <v>-390432</v>
+        <f>AVERAGE(D2:D26)</f>
       </c>
       <c r="E27" s="1">
-        <f t="shared" si="0"/>
-        <v>1.3099999999999997E-3</v>
+        <f>AVERAGE(E2:E26)</f>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="34.142857142857146" customWidth="1"/>
+    <col min="3" max="26" width="13.571428571428571" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2"/>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>